<commit_message>
Indicator 3 complete inc manual
</commit_message>
<xml_diff>
--- a/docs/tables/Various.xlsx
+++ b/docs/tables/Various.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ETest\docs\tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\EcoTest\docs\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E099F367-2E0F-4450-B8BB-32E878A52775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36F82E6E-6133-4E31-9A0C-65E4D591A6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{EE4263A2-8FC9-4695-B2B5-F7B8177F316B}"/>
+    <workbookView xWindow="1098" yWindow="1098" windowWidth="18300" windowHeight="12618" xr2:uid="{EE4263A2-8FC9-4695-B2B5-F7B8177F316B}"/>
   </bookViews>
   <sheets>
     <sheet name="Features" sheetId="15" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="88">
   <si>
     <t>Description</t>
   </si>
@@ -140,183 +140,9 @@
     <t>The ratio of length at 50% maturity (spawning fraction) to asymptotic length (von B. L-infinity)</t>
   </si>
   <si>
-    <t>I_rel</t>
-  </si>
-  <si>
     <t>Feature</t>
   </si>
   <si>
-    <t>The ratio of current index level to mean historical index level</t>
-  </si>
-  <si>
-    <t>I_g5</t>
-  </si>
-  <si>
-    <t>The slope in log index over the most recent 5 years</t>
-  </si>
-  <si>
-    <t>I_g10</t>
-  </si>
-  <si>
-    <t>The slope in log index over the most recent 10 years</t>
-  </si>
-  <si>
-    <t>I_g20</t>
-  </si>
-  <si>
-    <t>The slope in log index over the most recent 20 years</t>
-  </si>
-  <si>
-    <t>Isd1</t>
-  </si>
-  <si>
-    <t>Isd2</t>
-  </si>
-  <si>
-    <t>Isd3</t>
-  </si>
-  <si>
-    <t>As Isd1 but ENP of 20%</t>
-  </si>
-  <si>
-    <t>As Isd1 but ENP of 10%</t>
-  </si>
-  <si>
-    <t>C_rel</t>
-  </si>
-  <si>
-    <t>The ratio of current catches relative to mean historical levels</t>
-  </si>
-  <si>
-    <t>The slope in log catches over the most recent 5 years</t>
-  </si>
-  <si>
-    <t>The slope in log catches over the most recent 10 years</t>
-  </si>
-  <si>
-    <t>The slope in log catches over the most recent 20 years</t>
-  </si>
-  <si>
-    <t>Csd1</t>
-  </si>
-  <si>
-    <t>Mean absolute residual error in a log CPUE index from a loess smoother with effective number of parameters of 40% index length</t>
-  </si>
-  <si>
-    <t>ML_rel</t>
-  </si>
-  <si>
-    <t>The slope in log of mean length of catches over the most recent 5 years</t>
-  </si>
-  <si>
-    <t>The slope in log of mean length of catches over the most recent 10 years</t>
-  </si>
-  <si>
-    <t>The slope in log mean length of catches over the most recent 20 years</t>
-  </si>
-  <si>
-    <t>Standard deviation in residual error around log catches from a loess smoother with ENP 20% catch series length</t>
-  </si>
-  <si>
-    <t>MV_g5</t>
-  </si>
-  <si>
-    <t>ML_g5</t>
-  </si>
-  <si>
-    <t>ML_g10</t>
-  </si>
-  <si>
-    <t>ML_g20</t>
-  </si>
-  <si>
-    <t>MV_rel</t>
-  </si>
-  <si>
-    <t>MV_g10</t>
-  </si>
-  <si>
-    <t>MV_g20</t>
-  </si>
-  <si>
-    <t>ML_Linf</t>
-  </si>
-  <si>
-    <t>The ratio of current mean length in catches relative to asymptotic length (von B. L-infinity)</t>
-  </si>
-  <si>
-    <t>ML_L50</t>
-  </si>
-  <si>
-    <t>FM_rel</t>
-  </si>
-  <si>
-    <t>The ratio of current fraction mature fish in catches relative to historical mean fraction of mature fish in catches</t>
-  </si>
-  <si>
-    <t>The slope in log of fraction mature fish in catches over the most recent 5 years</t>
-  </si>
-  <si>
-    <t>The slope in log of fraction mature fish in catches over the most recent 10 years</t>
-  </si>
-  <si>
-    <t>The slope in log fraction mature fish in catches over the most recent 20 years</t>
-  </si>
-  <si>
-    <t>CR_mu</t>
-  </si>
-  <si>
-    <t>CR</t>
-  </si>
-  <si>
-    <t>The current catch ratio (first stock divided by second stock). R(y) = C(1,y) / C(2,y). CR is R from the most recent year, R(ny)</t>
-  </si>
-  <si>
-    <t>The catch ratio (first stock divided by second stock) over the first 20 years R[1:20]</t>
-  </si>
-  <si>
-    <t>CR_rel</t>
-  </si>
-  <si>
-    <t>CR / CR_mu</t>
-  </si>
-  <si>
-    <t>CR_s5</t>
-  </si>
-  <si>
-    <t>The slope in log CR over the most recent 5 years</t>
-  </si>
-  <si>
-    <t>CR_s10</t>
-  </si>
-  <si>
-    <t>The slope in log CR over the most recent 10 years</t>
-  </si>
-  <si>
-    <t>CC20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Correlation of the in residual fit of a loess smoother to log catches with ENP = 20% among stocks over the most recent 20 years. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">As CC20 but over historical years between 21 and 40 years ago. </t>
-  </si>
-  <si>
-    <t>CC60</t>
-  </si>
-  <si>
-    <t>CC40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As CC20 but over historical years between 41 and 60 years ago. </t>
-  </si>
-  <si>
-    <t>L5</t>
-  </si>
-  <si>
-    <t>LFS</t>
-  </si>
-  <si>
     <t>VML</t>
   </si>
   <si>
@@ -329,63 +155,12 @@
     <t>The shortest length at 5% selectivity phrased as a % of asymptotic length (L-infinity)</t>
   </si>
   <si>
-    <t>The ratio of current mean length in catches relative to historical average mean length in catches. Mean length is phrased as a % of asymptotic length (L-infinity)</t>
-  </si>
-  <si>
-    <t>The standard deviation in observed caught lengths in the current year relative to the historical average.</t>
-  </si>
-  <si>
-    <t>The slope in log standard deviation in catches over the most recent 5 years</t>
-  </si>
-  <si>
-    <t>The ratio of current mean length in cathes to length at 50% maturity (spawning fraction)</t>
-  </si>
-  <si>
-    <t>The slope in log standard deviation in catches over the most recent 10 years</t>
-  </si>
-  <si>
-    <t>The slope in log standard deviation in catches over the most recent 20 years</t>
-  </si>
-  <si>
     <t>Add magnitude of catches among fleets</t>
   </si>
   <si>
     <t>some indicator of overall impact of each fleet</t>
   </si>
   <si>
-    <t>C_g5</t>
-  </si>
-  <si>
-    <t>C_g10</t>
-  </si>
-  <si>
-    <t>C_g20</t>
-  </si>
-  <si>
-    <t>MA_rel</t>
-  </si>
-  <si>
-    <t>MA_g5</t>
-  </si>
-  <si>
-    <t>MA_g10</t>
-  </si>
-  <si>
-    <t>MA_g20</t>
-  </si>
-  <si>
-    <t>The ratio of current mean age in catch relative to mean historical levels</t>
-  </si>
-  <si>
-    <t>The slope in log mean age in catch over the most recent 5 years</t>
-  </si>
-  <si>
-    <t>The slope in log mean age in catch over the most recent 10 years</t>
-  </si>
-  <si>
-    <t>The slope in log mean age in catch over the most recent 20 years</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -398,10 +173,124 @@
     <t>Data</t>
   </si>
   <si>
-    <t>CF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The fraction of total historical catches (taken by this fleet). </t>
+    <t>L5_L50</t>
+  </si>
+  <si>
+    <t>LFS_L50</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>ML</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>MV</t>
+  </si>
+  <si>
+    <t>FM</t>
+  </si>
+  <si>
+    <t>_T</t>
+  </si>
+  <si>
+    <t>_Fleet1</t>
+  </si>
+  <si>
+    <t>_Fleet2</t>
+  </si>
+  <si>
+    <t>_Fleet3</t>
+  </si>
+  <si>
+    <t>Subscript</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>I_1_T</t>
+  </si>
+  <si>
+    <t>I_30_T</t>
+  </si>
+  <si>
+    <t>I_40_T</t>
+  </si>
+  <si>
+    <t>Total, all fleets combined</t>
+  </si>
+  <si>
+    <t>Fleet 1 (primary fleet)</t>
+  </si>
+  <si>
+    <t>Fleet 2 (secondary fleet)</t>
+  </si>
+  <si>
+    <t>Fleet 3 (all other fleets combined)</t>
+  </si>
+  <si>
+    <t>Relative biomass index (total) for first interpolation (oldest data point)</t>
+  </si>
+  <si>
+    <t>Relative biomass index (total) for 30th interpolation</t>
+  </si>
+  <si>
+    <t>Relative biomass index (total) for 40th interpolation (newest data point)</t>
+  </si>
+  <si>
+    <t>I_40_f1</t>
+  </si>
+  <si>
+    <t>C_2_f1</t>
+  </si>
+  <si>
+    <t>FM_11_f3</t>
+  </si>
+  <si>
+    <t>Relative vulnerable biomass index (fleet 1) for 40th interpolatin (newest data point)</t>
+  </si>
+  <si>
+    <t>Catch relative to historical mean</t>
+  </si>
+  <si>
+    <t>Mean length in catches relative to historical mean</t>
+  </si>
+  <si>
+    <t>Mean age in catches relative to maximum age (maxa)</t>
+  </si>
+  <si>
+    <t>Coefficient of variation in catch lengths</t>
+  </si>
+  <si>
+    <t>Fraction mature fish in catch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Index of biomass (_T) or vulnerable biomass (_f1, _f2, _f3) relative to historical mean. </t>
+  </si>
+  <si>
+    <t>Catch for fleet 1 in the first interpolation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fraction mature fish in fleet 3 catches in interpolation 11. </t>
+  </si>
+  <si>
+    <t>Csd</t>
+  </si>
+  <si>
+    <t>Isd</t>
+  </si>
+  <si>
+    <t>The variability in catches around a smoother (internal function)</t>
+  </si>
+  <si>
+    <t>The variability in relative abundance indices around a smoother (internal function)</t>
   </si>
 </sst>
 </file>
@@ -476,9 +365,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -516,7 +405,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -622,7 +511,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -764,7 +653,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -772,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C8A4713-AE3F-47AB-A996-17263352EFC5}">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="2" width="11.5234375" customWidth="1"/>
@@ -781,10 +670,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>119</v>
+        <v>44</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -795,7 +684,7 @@
         <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
         <v>30</v>
@@ -806,7 +695,7 @@
         <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s">
         <v>32</v>
@@ -817,7 +706,7 @@
         <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
@@ -828,7 +717,7 @@
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
@@ -836,189 +725,189 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>121</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>121</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>121</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>97</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>84</v>
       </c>
       <c r="B9" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" t="s">
         <v>47</v>
       </c>
-      <c r="B14" t="s">
-        <v>122</v>
-      </c>
       <c r="C14" t="s">
-        <v>49</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>122</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
-        <v>108</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>122</v>
+        <v>60</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
-        <v>109</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
-        <v>122</v>
+        <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>122</v>
+        <v>60</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B20" t="s">
-        <v>122</v>
+        <v>60</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>122</v>
+        <v>61</v>
       </c>
       <c r="C21" t="s">
-        <v>124</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B22" t="s">
-        <v>122</v>
+        <v>61</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.55000000000000004">
@@ -1026,274 +915,43 @@
         <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>122</v>
+        <v>61</v>
       </c>
       <c r="C23" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B24" t="s">
-        <v>122</v>
+        <v>61</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B25" t="s">
-        <v>122</v>
+        <v>61</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" t="s">
-        <v>72</v>
-      </c>
-      <c r="B27" t="s">
-        <v>122</v>
-      </c>
-      <c r="C27" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" t="s">
-        <v>111</v>
-      </c>
-      <c r="B28" t="s">
-        <v>122</v>
-      </c>
-      <c r="C28" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" t="s">
-        <v>112</v>
-      </c>
-      <c r="B29" t="s">
-        <v>122</v>
-      </c>
-      <c r="C29" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" t="s">
-        <v>113</v>
-      </c>
-      <c r="B30" t="s">
-        <v>122</v>
-      </c>
-      <c r="C30" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" t="s">
-        <v>114</v>
-      </c>
-      <c r="B31" t="s">
-        <v>122</v>
-      </c>
-      <c r="C31" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" t="s">
-        <v>67</v>
-      </c>
-      <c r="B32" t="s">
-        <v>122</v>
-      </c>
-      <c r="C32" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" t="s">
-        <v>63</v>
-      </c>
-      <c r="B33" t="s">
-        <v>122</v>
-      </c>
-      <c r="C33" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" t="s">
-        <v>122</v>
-      </c>
-      <c r="C34" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" t="s">
-        <v>69</v>
-      </c>
-      <c r="B35" t="s">
-        <v>122</v>
-      </c>
-      <c r="C35" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" t="s">
-        <v>73</v>
-      </c>
-      <c r="B36" t="s">
-        <v>122</v>
-      </c>
-      <c r="C36" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" t="s">
-        <v>63</v>
-      </c>
-      <c r="B37" t="s">
-        <v>122</v>
-      </c>
-      <c r="C37" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" t="s">
-        <v>68</v>
-      </c>
-      <c r="B38" t="s">
-        <v>122</v>
-      </c>
-      <c r="C38" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" t="s">
-        <v>69</v>
-      </c>
-      <c r="B39" t="s">
-        <v>122</v>
-      </c>
-      <c r="C39" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" t="s">
-        <v>79</v>
-      </c>
-      <c r="B40" t="s">
-        <v>122</v>
-      </c>
-      <c r="C40" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" t="s">
-        <v>78</v>
-      </c>
-      <c r="B41" t="s">
-        <v>122</v>
-      </c>
-      <c r="C41" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" t="s">
-        <v>82</v>
-      </c>
-      <c r="B42" t="s">
-        <v>122</v>
-      </c>
-      <c r="C42" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" t="s">
-        <v>84</v>
-      </c>
-      <c r="B43" t="s">
-        <v>122</v>
-      </c>
-      <c r="C43" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" t="s">
-        <v>86</v>
-      </c>
-      <c r="B44" t="s">
-        <v>122</v>
-      </c>
-      <c r="C44" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" t="s">
-        <v>88</v>
-      </c>
-      <c r="B45" t="s">
-        <v>122</v>
-      </c>
-      <c r="C45" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" t="s">
-        <v>92</v>
-      </c>
-      <c r="B46" t="s">
-        <v>122</v>
-      </c>
-      <c r="C46" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" t="s">
-        <v>91</v>
-      </c>
-      <c r="B47" t="s">
-        <v>122</v>
-      </c>
-      <c r="C47" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1320,10 +978,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>